<commit_message>
Add T303 folder management (F4) and verify on real device
Adds folder CRUD/stats/merge/item-move to the repository, root and
subfolder screens with a bottom-nav "도감/폴더" tab shell, and folder
pickers wired into the register form and item detail screen.

Real-device testing surfaced two bugs: the folder picker sheet
returned null for both "dismissed" and "unclassified selected"
(fixed with an empty-string sentinel), and the folder tab's stats
went stale because IndexedStack keeps it alive across tab switches
(fixed by keying it to a counter bumped on every item change).

Also updates PROGRESS.md and the roadmap spreadsheet — Phase 1 is
now fully complete through T303.
</commit_message>
<xml_diff>
--- a/pong_dang_project_roadmap.xlsx
+++ b/pong_dang_project_roadmap.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>진행중 (T301/T302 완료, T303 진행 예정)</t>
+          <t>완료</t>
         </is>
       </c>
     </row>
@@ -1103,19 +1103,19 @@
         </is>
       </c>
       <c r="F13" s="13" t="n">
-        <v>46215</v>
+        <v>46214</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>46218</v>
+        <v>46214</v>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>대기</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>폴더 이동 및 트랙 구조 UI 컴포넌트 구현 — [실제] (일정 조정) T302 완료 다음날로 시작일 당김, 추정 소요일수(4일)는 원안 유지</t>
+          <t>폴더 이동 및 트랙 구조 UI 컴포넌트 구현 — [실제] (일정 조정) T302 완료 다음날로 시작일 당김, 추정 소요일수(4일)는 원안 유지 / [실제] 폴더 CRUD+통계+병합+아이템이동 구현, 실기기에서 생성/이동/통계갱신 검증</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add T401 calendar UI and Phase 2 feature spec
Writes docs/T401_phase2_feature_spec.md (F7-F9) from the original
planning PDF before implementing, per the T101 precedent, then adds
deco_entries/deco_placements schema (with a v1->v2 migration) and the
self-built month calendar with per-day entry indicators.

Real-device testing plus user feedback drove two design changes:
entries are no longer created just by opening a day (only on actual
save), and the save button is disabled when there's nothing new to
persist. Also fixes a repeat of the same setState/Future bug from
T302, this time in CalendarScreen._reload().
</commit_message>
<xml_diff>
--- a/pong_dang_project_roadmap.xlsx
+++ b/pong_dang_project_roadmap.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>대기</t>
+          <t>진행중 (T401 완료, T402 진행 예정)</t>
         </is>
       </c>
     </row>
@@ -1141,19 +1141,19 @@
         </is>
       </c>
       <c r="F14" s="14" t="n">
-        <v>46232</v>
+        <v>46214</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>46234</v>
+        <v>46214</v>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>대기</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>table_calendar 패키지 커스텀 가이드 요청 — [참고] T303 이후(Phase 2/3) 날짜는 원안 그대로 유지된 추정치입니다. T303 진행 상황을 보고 재산정 필요</t>
+          <t>table_calendar 패키지 커스텀 가이드 요청 — [참고] T303 이후(Phase 2/3) 날짜는 원안 그대로 유지된 추정치입니다. T303 진행 상황을 보고 재산정 필요 / [실제] table_calendar 없이 자체 구현. T101처럼 사전 상세 명세서(T401_phase2_feature_spec.md) 작성 후 구현. 실기기 검증 완료</t>
         </is>
       </c>
     </row>
@@ -1179,10 +1179,10 @@
         </is>
       </c>
       <c r="F15" s="13" t="n">
-        <v>46235</v>
+        <v>46215</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>46239</v>
+        <v>46219</v>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
@@ -1217,10 +1217,10 @@
         </is>
       </c>
       <c r="F16" s="14" t="n">
-        <v>46240</v>
+        <v>46220</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>46242</v>
+        <v>46222</v>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>

</xml_diff>